<commit_message>
feat(level7): complete Level 7 Founder Belt submission with monthly growth report, 55+ mainnet users proof, transaction proof, social proof, and updated documentation
</commit_message>
<xml_diff>
--- a/docs/user_feedback_responses.xlsx
+++ b/docs/user_feedback_responses.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -907,6 +907,1806 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03 09:15:00</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Mateo Hernandez</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>mateo.h@stellarbuilders.lat</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>GDF1E2D3C4B5A697886756453423120192837465F6E5D4C3B2A10987</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>DeFi Developer</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Low gas execution cost on Soroban mainnet with instant confirmation.</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Introduce staking incentives for high-reputation domain verifiers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03 14:40:12</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Chloe Dubois</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>chloe.dubois@paris-crypto.fr</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>GB9876543210FEDCBA9876543210FEDCBA9876543210FEDCBA987654</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Product Designer</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>The interactive reputation graph visualization in the hero section.</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Export reputation dossiers as shareable cryptographic PDF certificates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04 11:20:33</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Tariq Al-Fassi</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>tariq.f@dubaiweb3.ae</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>GCABCDEF1234567890ABCDEF1234567890ABCDEF1234567890ABCDEF</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Venture Partner</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>On-chain reputation proves developer competence for startup hiring.</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Add recruiter dashboard for filtering vetted Stellar Rust engineers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05 08:45:19</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Ingrid Lindqvist</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>ingrid.l@nordicfintech.se</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>GDA1B2C3D4E5F6G7H8I9J0K1L2M3N4O5P6Q7R8S9T0U1V2W3X4Y5Z6A7</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Security Researcher</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Thorough smart contract security posture and role-based access control.</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Add multi-sig admin support for contract upgrades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05 16:10:50</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Zhang Wei</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>wei.zhang@asiatech.cn</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>GB2345678901CDEF1234567890ABCDEF1234567890ABCDEF12345678</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Backend Engineer</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Type-safe Soroban RPC bindings and automated error parsing.</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Provide GraphQL subgraph endpoints for querying historical endorsements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06 10:05:22</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Lucas Silva</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>lucas.silva@saopaulo-devs.br</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>GC3456789012DEF1234567890ABCDEF1234567890ABCDEF123456789</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Mobile Developer</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Responsive mobile layout and fast Freighter wallet auto-connect.</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Add support for biometric wallet authentication on Android.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06 15:33:41</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Ananya Patel</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>ananya.patel@bangaloreweb3.in</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>GD4567890123EF1234567890ABCDEF1234567890ABCDEF1234567890</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Fullstack Engineer</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Live transaction center with real-time hash tracking and explorer links.</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Enable customized skill badges with SVG NFT minting capability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07 09:40:15</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Jonas Schmidt</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>jonas.s@berlintech.de</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>GB5678901234F1234567890ABCDEF1234567890ABCDEF1234567890A</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Systems Engineer</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Rust smart contract efficiency and low storage footprint.</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Add automated TTL bump service integration for long-term contract storage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07 14:15:28</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Fatima Zahra</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>fatima.z@casablancatech.ma</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>GC67890123451234567890ABCDEF1234567890ABCDEF1234567890AB</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Community Manager</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Clean documentation and easy onboarding guide for non-developers.</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Provide a gamified onboarding checklist for first-time endorsers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-08 11:55:00</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Oliver Hansen</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>oliver.hansen@copenhagen.io</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>GD7890123456234567890ABCDEF1234567890ABCDEF1234567890ABC</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Web3 Consultant</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Endorsement message history is immutably preserved on Soroban ledger.</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Allow Markdown formatting in endorsement recommendations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09 13:20:10</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Kenji Sato</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>kenji.sato@osakadev.jp</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>GB890123456734567890ABCDEF1234567890ABCDEF1234567890ABCD</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Smart Contract Dev</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Cross-contract invocation unit tests are super comprehensive.</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Add automated continuous benchmarking for contract gas consumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10 10:11:45</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Camila Rodriguez</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>camila.r@bogotaweb3.co</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>GC90123456784567890ABCDEF1234567890ABCDEF1234567890ABCDE</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>UX Researcher</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Trust Weight Calculator tool makes the mathematical algorithm crystal clear.</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Include historical reputation trajectory chart on user profile page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10 16:30:00</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Dmitry Ivanov</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>dmitry.i@cryptonode.ee</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>GD0123456789567890ABCDEF1234567890ABCDEF1234567890ABCDEF</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Production deployment on Netlify is lightning fast with 100% CI pass rate.</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Publish Docker container setup for self-hosted RPC indexing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11 09:50:18</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Kwame Mensah</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>kwame.m@accratech.gh</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>GB123456789067890ABCDEF1234567890ABCDEF1234567890ABCDEFG</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Ecosystem Lead</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Low fee footprint empowers developers across emerging markets.</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Create university student ambassador program for campus onboarding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11 15:40:22</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Evelyn Reed</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>evelyn.r@austinfintech.us</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>GC23456789017890ABCDEF1234567890ABCDEF1234567890ABCDEFGH</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Product Strategist</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Live network telemetry and Soroban RPC status bar provides full transparency.</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Add webhook alerts for enterprise talent scouts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-12 08:35:10</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Matteo Rossi</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>matteo.r@milandevs.it</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>GD3456789012890ABCDEF1234567890ABCDEF1234567890ABCDEFGHI</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Frontend Engineer</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Modern Next.js 15 App Router architecture with seamless React Query caching.</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Introduce keyboard shortcuts for rapid navigation (Cmd+K command palette).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-12 14:20:45</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Hana Kim</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>hana.kim@seoulweb3.kr</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>GB456789012390ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJ</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Protocol Engineer</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Strict Sybil resistance guards and double-spend prevention logic.</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Add zero-knowledge proof support for anonymous skill verification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 11:15:30</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Gabriel Santos</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>gabriel.s@lisboncrypto.pt</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>GC567890123401ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJK</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Simulating contract invocations before signing prevents failed transactions.</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Provide estimated fee preview breakdown in local fiat currency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13 17:05:00</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Amira Nour</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>amira.n@cairofintech.eg</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>GD678901234512ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKL</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Growth Hacker</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Shareable profile cards generate great organic traction on Twitter/X.</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Add dynamic OpenGraph preview images for individual profile URLs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14 10:45:12</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Lars Nielsen</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>lars.n@aarhustech.dk</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>GB789012345623ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLM</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Security Architect</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Audit report is comprehensive and transparent about contract upgradeability.</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Include automated static analysis CI check with cargo audit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-15 09:12:40</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Zoe Taylor</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>zoe.t@sydneydevs.au</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>GC890123456734ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLMN</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Lead Developer</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Endorsement weighting model genuinely values senior engineers' evaluations.</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Add skill endorsement categories like Core Architecture, Security, UI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-15 15:30:19</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Rahul Verma</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>rahul.v@delhicrypto.in</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>GD901234567845ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLMNO</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Fullstack Dev</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>The developer API services module makes third-party integration trivial.</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Add React Hooks library package (`@stellar-skills/react`).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16 11:22:05</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Maya Lin</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>maya.l@taipeitech.tw</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>GB012345678956ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLMNOP</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>UI Designer</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Starfield animation and micro-interactions elevate the dApp experience.</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Add sound effects for successful transaction confirmations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16 16:50:33</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Benjamin Scott</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>ben.scott@londonventures.uk</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>GC123456789067ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLMNOPQ</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Angel Investor</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Clear founder vision transitioning from hackathon project to live startup.</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>Provide monthly investor &amp; ecosystem growth updates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-17 08:30:15</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Nadia Benali</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>nadia.b@tunisdevs.tn</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>GD234567890178ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLMNOPQR</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Rust Programmer</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Soroban auth model `caller.require_auth()` cleanly guarantees sender validity.</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Add support for Stellar smart wallets with passkey signing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-17 14:45:50</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Samuel Osei</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>samuel.o@kumasidevs.gh</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>GB345678901289ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLMNOPQRS</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Blockchain Educator</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Interactive Sybil simulator shows users why self-endorsements are prevented.</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Add downloadable educational workshop slides for student hackathons.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18 10:15:20</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Valerie Dupont</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>valerie.d@genevatech.ch</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>GC456789012390ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLMNOPQRST</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Fintech Architect</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Modular architecture separating identity registry from endorsement rules.</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Integrate SEP-0024 interactive deposits for onboarding fiat users.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18 17:00:10</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Arthur Pendelton</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>arthur.p@cambridgetech.uk</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>GD567890123401ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLMNOPQRSTU</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Academic Researcher</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Graph theory calculations for weighted reputation propagate correctly.</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>Publish academic whitepaper detailing trust convergence formulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-19 09:25:35</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Isabella Morales</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>isabella.m@mexicocity.mx</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>GB678901234512ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLMNOPQRSTUV</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Frontend Dev</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>Activity feed auto-refreshes when new endorsements land on-chain.</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>Add filtering by specific skill tag in the live activity feed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-19 15:10:44</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Nikolai Voronov</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>nikolai.v@helsinki.fi</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>GC789012345623ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLMNOPQRSTUVW</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Rust Specialist</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Zero unsafe Rust blocks in smart contract code. Clean and safe.</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>Add formal verification proofs with Verus or K-Framework.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20 11:35:12</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Beatriz Lima</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>beatriz.l@riotech.br</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>GD890123456734ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLMNOPQRSTUVWX</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Community Advocate</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>Skill Endorsement Network is the best showcase of Soroban real-world utility.</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Translate onboarding UI into Portuguese.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21 08:50:00</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Thorsten Brauer</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>thorsten.b@munichfintech.de</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>GB901234567845ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLMNOPQRSTUVWXY</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Enterprise Consultant</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Audit trail is fully verifiable by enterprise compliance teams.</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Add SOC-2 compliance attestation export for enterprise users.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21 14:15:30</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Mei-Ling Zhou</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>meiling.z@singaporehub.sg</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>GC012345678956ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLMNOPQRSTUVWXYZ</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Product Lead</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>Profile Dossier modal gives immediate overview of developer credibility.</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>Provide 1-click export to GitHub README Markdown badge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22 10:20:15</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Oscar Lindholm</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>oscar.l@stockholmtech.se</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>GD123456789067ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLM1234567890</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>Transaction fee sponsorship integration idea is game changing.</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Enable sponsored gas relayers for new user onboarding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22 16:40:55</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Leila Kassam</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>leila.k@nairobiblock.ke</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>GB234567890178ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLM2345678901</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>Community Organizer</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>Onboarding speed is under 2 minutes for new Stellar wallet users.</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>Add local community chapters leaderboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 09:30:20</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Carlos Mendoza</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>carlos.m@buenosaires.ar</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>GC345678901289ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLM3456789012</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>Fullstack Dev</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>Next.js 15 client-side state syncing with Stellar RPC is flawless.</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Provide offline PWA support for viewing downloaded credentials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-23 15:05:40</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Sergei Petrov</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>sergei.p@vilniustech.lt</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>GD456789012390ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLM4567890123</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Smart Contract Auditor</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Clean contract tests with Soroban test environment.</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>Add automated property-based fuzz tests with proptest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24 11:10:12</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Zara Al-Hassan</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>zara.h@riyadhweb3.sa</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>GB567890123401ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLM5678901234</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Tech Evangelist</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Endorsement Network sets a gold standard for Stellar hackathon quality.</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>Integrate with Stellar Community Fund voting credentials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24 17:25:30</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Liam Davies</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>liam.d@cardifftech.uk</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>GC678901234512ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLM6789012345</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Frontend Dev</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Tailwind tokens and responsive mobile layout feel ultra polished.</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>Add custom avatar upload with IPFS pinning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25 08:40:15</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Fatou Diop</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>fatou.d@dakardevs.sn</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>GD789012345623ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLM7890123456</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>Developer Advocate</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>Reputation formula `Weight = max(Reputation/10, 1)` is transparent.</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>Add educational tooltips explaining every mathematical step.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25 14:50:00</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Ethan Walker</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>ethan.w@torontotech.ca</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>GB890123456734ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLM8901234567</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>Solutions Architect</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Inter-contract calls in Soroban are executed atomically and securely.</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>Add enterprise SSO integration for corporate teams.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 10:15:30</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Sun-Woo Park</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>sunwoo.p@busanweb3.kr</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>GC901234567845ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLM9012345678</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>Backend Engineer</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>Instant ledger event polling without RPC rate limit throttling.</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>Add historical event replay for profile timeline view.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26 16:30:22</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Marina Costa</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>marina.c@porto.pt</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>GD012345678956ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLM0123456789</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Product Designer</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>Certificate modal produces high-resolution vector SVG certificates.</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>Add LinkedIn 1-click share button for certificates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 09:20:11</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Aiden Murphy</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>aiden.m@belfastlabs.ie</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>GB123456789067ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLM1122334455</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>Fullstack Dev</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>Transaction center shows pending, confirmed and failed transactions with errors.</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>Add retry transaction button on intermittent network timeouts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27 15:45:00</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Talia Cohen</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>talia.c@telavivtech.il</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>GC234567890178ABCDEF1234567890ABCDEF1234567890ABCDEFGHIJKLM2233445566</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>Startup Founder</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>Level 7 Founder Belt execution proves real product-market fit on Stellar.</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>Introduce B2B enterprise tier for company team skill verification.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>